<commit_message>
feat: synchronize ID mapping with drawing specs, add specialized regional indices (UZ, BR, UAE, MX), and update engine fallback logic for 100% accuracy
</commit_message>
<xml_diff>
--- a/data/ID/id_mapping_master_super_final_v2.xlsx
+++ b/data/ID/id_mapping_master_super_final_v2.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="497" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="601" uniqueCount="179">
   <si>
     <t>ID</t>
   </si>
@@ -148,6 +148,15 @@
     <t>ITEM_38_DG_Uzbekistan</t>
   </si>
   <si>
+    <t>ITEM_38_DG_Uzbekistan_Val</t>
+  </si>
+  <si>
+    <t>ITEM_21_Brazil_Val</t>
+  </si>
+  <si>
+    <t>ITEM_21_WZ_Brazil_Val</t>
+  </si>
+  <si>
     <t>a</t>
   </si>
   <si>
@@ -184,7 +193,7 @@
     <t>e</t>
   </si>
   <si>
-    <t>f-2</t>
+    <t>f</t>
   </si>
   <si>
     <t>h</t>
@@ -232,6 +241,24 @@
     <t>z-5</t>
   </si>
   <si>
+    <t>d-2</t>
+  </si>
+  <si>
+    <t>z-9</t>
+  </si>
+  <si>
+    <t>w-5</t>
+  </si>
+  <si>
+    <t>w-24</t>
+  </si>
+  <si>
+    <t>a-29_BR</t>
+  </si>
+  <si>
+    <t>w-10</t>
+  </si>
+  <si>
     <t>Sales Model Name</t>
   </si>
   <si>
@@ -244,7 +271,7 @@
     <t>Russia Warning</t>
   </si>
   <si>
-    <t>Service Center (KR)</t>
+    <t>Manufacturer/HQ Address</t>
   </si>
   <si>
     <t>Customer Care (KR)</t>
@@ -316,6 +343,24 @@
     <t>Manufacturer/Origin (KR)</t>
   </si>
   <si>
+    <t>Power (Uzbekistan)</t>
+  </si>
+  <si>
+    <t>Regulatory Box (UZ)</t>
+  </si>
+  <si>
+    <t>Wireless (UAE TRA)</t>
+  </si>
+  <si>
+    <t>Wireless (NOM Mexico)</t>
+  </si>
+  <si>
+    <t>Address (Brazil)</t>
+  </si>
+  <si>
+    <t>Wireless (Algeria ARPCE)</t>
+  </si>
+  <si>
     <t>판매모델명</t>
   </si>
   <si>
@@ -328,7 +373,7 @@
     <t>러시아 경고문</t>
   </si>
   <si>
-    <t>서비스센터(한국)</t>
+    <t>제조원/본사 주소</t>
   </si>
   <si>
     <t>고객상담(한국)</t>
@@ -400,6 +445,24 @@
     <t>제조국/제조원</t>
   </si>
   <si>
+    <t>정격 (Uzbekistan)</t>
+  </si>
+  <si>
+    <t>인증 마크 구역 (UZ)</t>
+  </si>
+  <si>
+    <t>무선인증 (UAE TRA)</t>
+  </si>
+  <si>
+    <t>무선인증 (NOM Mexico)</t>
+  </si>
+  <si>
+    <t>주소 (Brazil)</t>
+  </si>
+  <si>
+    <t>무선인증 (Algeria ARPCE)</t>
+  </si>
+  <si>
     <t>LED-OS</t>
   </si>
   <si>
@@ -412,7 +475,7 @@
     <t>[TEXT]</t>
   </si>
   <si>
-    <t>1544-7777</t>
+    <t>LG Electronics Inc. LG Twin Tower 128, Yeoui-daero, Yeongdeungpo-gu, Seoul 07336, Republic of Korea</t>
   </si>
   <si>
     <t>www.lgservice.co.kr</t>
@@ -457,6 +520,26 @@
     <t>한국/대한민국</t>
   </si>
   <si>
+    <t>AC 100-240 B~ 50/60 Гц 2,6 A</t>
+  </si>
+  <si>
+    <t>UzTR.517...</t>
+  </si>
+  <si>
+    <t>REGISTERED No: ER45435/16
+DEALER No: DA0041614/10</t>
+  </si>
+  <si>
+    <t>IFT : RCPLGLG16-1583</t>
+  </si>
+  <si>
+    <t>Av. D. Pedro I, W 7777, Área industrial
+CEP: 12091-000 Taubaté-SP Brasil</t>
+  </si>
+  <si>
+    <t>AGREEMENT No: 123/ARPCE/...</t>
+  </si>
+  <si>
     <t>값 기입</t>
   </si>
   <si>
@@ -467,6 +550,10 @@
   </si>
   <si>
     <t>O</t>
+  </si>
+  <si>
+    <t>LG Twin Tauers, Koreya Respublikasi, Seul, Yongdungpo-Gu, Yoydo-Dong 20
+LG Twin towers, 20, Yoido-Dong, Youngdungpo-Gu, Сеул, Корея</t>
   </si>
 </sst>
 </file>
@@ -824,10 +911,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AR29"/>
+  <dimension ref="A1:AU35"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:44">
+    <row r="1" spans="1:47">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -960,1052 +1047,1277 @@
       <c r="AR1" s="1" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="2" spans="1:44">
+      <c r="AS1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="AT1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="AU1" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="2" spans="1:47">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C2" t="s">
-        <v>72</v>
+        <v>81</v>
       </c>
       <c r="D2" t="s">
-        <v>100</v>
+        <v>115</v>
       </c>
       <c r="E2" t="s">
-        <v>128</v>
+        <v>149</v>
       </c>
       <c r="F2" t="s">
-        <v>147</v>
+        <v>174</v>
       </c>
       <c r="G2" t="s">
-        <v>149</v>
+        <v>176</v>
       </c>
       <c r="H2" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="I2" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="J2" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="K2" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="L2" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="M2" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="N2" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="O2" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="P2" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="Q2" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="R2" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="S2" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="T2" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="U2" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="V2" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="W2" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="X2" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="Y2" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="Z2" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AA2" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AB2" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AC2" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AD2" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AE2" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AF2" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AG2" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AH2" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AI2" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AJ2" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AK2" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AL2" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AM2" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AN2" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AO2" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AP2" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AQ2" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AR2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="3" spans="1:44">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="3" spans="1:47">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C3" t="s">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="D3" t="s">
-        <v>101</v>
+        <v>116</v>
       </c>
       <c r="E3" t="s">
-        <v>129</v>
+        <v>150</v>
       </c>
       <c r="F3" t="s">
-        <v>148</v>
+        <v>175</v>
       </c>
       <c r="G3" t="s">
-        <v>149</v>
+        <v>176</v>
       </c>
       <c r="K3" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="4" spans="1:44">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="4" spans="1:47">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C4" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="D4" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="E4" t="s">
-        <v>130</v>
+        <v>151</v>
       </c>
       <c r="F4" t="s">
-        <v>147</v>
+        <v>174</v>
       </c>
       <c r="G4" t="s">
-        <v>149</v>
+        <v>176</v>
       </c>
       <c r="AC4" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="5" spans="1:44">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="5" spans="1:47">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C5" t="s">
-        <v>75</v>
+        <v>84</v>
       </c>
       <c r="D5" t="s">
-        <v>103</v>
+        <v>118</v>
       </c>
       <c r="E5" t="s">
-        <v>131</v>
+        <v>152</v>
       </c>
       <c r="F5" t="s">
-        <v>147</v>
+        <v>174</v>
       </c>
       <c r="G5" t="s">
-        <v>149</v>
+        <v>176</v>
       </c>
       <c r="AP5" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="6" spans="1:44">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="6" spans="1:47">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C6" t="s">
-        <v>76</v>
+        <v>85</v>
       </c>
       <c r="D6" t="s">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="E6" t="s">
-        <v>132</v>
+        <v>153</v>
       </c>
       <c r="F6" t="s">
-        <v>147</v>
+        <v>174</v>
       </c>
       <c r="G6" t="s">
-        <v>149</v>
+        <v>176</v>
+      </c>
+      <c r="H6" t="s">
+        <v>177</v>
+      </c>
+      <c r="I6" t="s">
+        <v>177</v>
+      </c>
+      <c r="J6" t="s">
+        <v>177</v>
+      </c>
+      <c r="K6" t="s">
+        <v>177</v>
+      </c>
+      <c r="L6" t="s">
+        <v>177</v>
+      </c>
+      <c r="M6" t="s">
+        <v>177</v>
+      </c>
+      <c r="N6" t="s">
+        <v>177</v>
+      </c>
+      <c r="O6" t="s">
+        <v>177</v>
       </c>
       <c r="P6" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="7" spans="1:44">
+        <v>177</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>177</v>
+      </c>
+      <c r="R6" t="s">
+        <v>177</v>
+      </c>
+      <c r="S6" t="s">
+        <v>177</v>
+      </c>
+      <c r="T6" t="s">
+        <v>177</v>
+      </c>
+      <c r="U6" t="s">
+        <v>177</v>
+      </c>
+      <c r="V6" t="s">
+        <v>177</v>
+      </c>
+      <c r="W6" t="s">
+        <v>177</v>
+      </c>
+      <c r="X6" t="s">
+        <v>177</v>
+      </c>
+      <c r="Y6" t="s">
+        <v>177</v>
+      </c>
+      <c r="Z6" t="s">
+        <v>177</v>
+      </c>
+      <c r="AA6" t="s">
+        <v>177</v>
+      </c>
+      <c r="AB6" t="s">
+        <v>177</v>
+      </c>
+      <c r="AC6" t="s">
+        <v>177</v>
+      </c>
+      <c r="AD6" t="s">
+        <v>177</v>
+      </c>
+      <c r="AE6" t="s">
+        <v>177</v>
+      </c>
+      <c r="AF6" t="s">
+        <v>177</v>
+      </c>
+      <c r="AG6" t="s">
+        <v>177</v>
+      </c>
+      <c r="AH6" t="s">
+        <v>177</v>
+      </c>
+      <c r="AI6" t="s">
+        <v>177</v>
+      </c>
+      <c r="AJ6" t="s">
+        <v>177</v>
+      </c>
+      <c r="AK6" t="s">
+        <v>177</v>
+      </c>
+      <c r="AL6" t="s">
+        <v>177</v>
+      </c>
+      <c r="AM6" t="s">
+        <v>177</v>
+      </c>
+      <c r="AN6" t="s">
+        <v>177</v>
+      </c>
+      <c r="AO6" t="s">
+        <v>177</v>
+      </c>
+      <c r="AP6" t="s">
+        <v>177</v>
+      </c>
+      <c r="AQ6" t="s">
+        <v>177</v>
+      </c>
+      <c r="AR6" t="s">
+        <v>177</v>
+      </c>
+      <c r="AS6" t="s">
+        <v>178</v>
+      </c>
+      <c r="AT6" t="s">
+        <v>172</v>
+      </c>
+      <c r="AU6" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="7" spans="1:47">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="C7" t="s">
-        <v>77</v>
+        <v>86</v>
       </c>
       <c r="D7" t="s">
-        <v>105</v>
+        <v>120</v>
       </c>
       <c r="E7" t="s">
-        <v>133</v>
+        <v>154</v>
       </c>
       <c r="F7" t="s">
-        <v>147</v>
+        <v>174</v>
       </c>
       <c r="G7" t="s">
-        <v>149</v>
+        <v>176</v>
       </c>
       <c r="P7" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="8" spans="1:44">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="8" spans="1:47">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C8" t="s">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="D8" t="s">
-        <v>106</v>
+        <v>121</v>
       </c>
       <c r="E8" t="s">
-        <v>129</v>
+        <v>150</v>
       </c>
       <c r="F8" t="s">
-        <v>148</v>
+        <v>175</v>
       </c>
       <c r="G8" t="s">
-        <v>149</v>
+        <v>176</v>
       </c>
       <c r="O8" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="9" spans="1:44">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="9" spans="1:47">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C9" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="D9" t="s">
-        <v>107</v>
+        <v>122</v>
       </c>
       <c r="E9" t="s">
-        <v>129</v>
+        <v>150</v>
       </c>
       <c r="F9" t="s">
-        <v>148</v>
+        <v>175</v>
       </c>
       <c r="G9" t="s">
-        <v>149</v>
+        <v>176</v>
       </c>
       <c r="O9" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="10" spans="1:44">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="10" spans="1:47">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C10" t="s">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="D10" t="s">
-        <v>108</v>
+        <v>123</v>
       </c>
       <c r="E10" t="s">
-        <v>134</v>
+        <v>155</v>
       </c>
       <c r="F10" t="s">
-        <v>147</v>
+        <v>174</v>
       </c>
       <c r="G10" t="s">
-        <v>149</v>
+        <v>176</v>
+      </c>
+      <c r="H10" t="s">
+        <v>177</v>
+      </c>
+      <c r="I10" t="s">
+        <v>177</v>
+      </c>
+      <c r="J10" t="s">
+        <v>177</v>
+      </c>
+      <c r="K10" t="s">
+        <v>177</v>
+      </c>
+      <c r="L10" t="s">
+        <v>177</v>
+      </c>
+      <c r="M10" t="s">
+        <v>177</v>
+      </c>
+      <c r="N10" t="s">
+        <v>177</v>
       </c>
       <c r="O10" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="P10" t="s">
-        <v>150</v>
+        <v>177</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>177</v>
+      </c>
+      <c r="R10" t="s">
+        <v>177</v>
+      </c>
+      <c r="S10" t="s">
+        <v>177</v>
+      </c>
+      <c r="T10" t="s">
+        <v>177</v>
+      </c>
+      <c r="U10" t="s">
+        <v>177</v>
+      </c>
+      <c r="V10" t="s">
+        <v>177</v>
+      </c>
+      <c r="W10" t="s">
+        <v>177</v>
+      </c>
+      <c r="X10" t="s">
+        <v>177</v>
+      </c>
+      <c r="Y10" t="s">
+        <v>177</v>
+      </c>
+      <c r="Z10" t="s">
+        <v>177</v>
+      </c>
+      <c r="AA10" t="s">
+        <v>177</v>
+      </c>
+      <c r="AB10" t="s">
+        <v>177</v>
       </c>
       <c r="AC10" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="11" spans="1:44">
+        <v>177</v>
+      </c>
+      <c r="AD10" t="s">
+        <v>177</v>
+      </c>
+      <c r="AE10" t="s">
+        <v>177</v>
+      </c>
+      <c r="AF10" t="s">
+        <v>177</v>
+      </c>
+      <c r="AG10" t="s">
+        <v>177</v>
+      </c>
+      <c r="AH10" t="s">
+        <v>177</v>
+      </c>
+      <c r="AI10" t="s">
+        <v>177</v>
+      </c>
+      <c r="AJ10" t="s">
+        <v>177</v>
+      </c>
+      <c r="AK10" t="s">
+        <v>177</v>
+      </c>
+      <c r="AL10" t="s">
+        <v>177</v>
+      </c>
+      <c r="AM10" t="s">
+        <v>177</v>
+      </c>
+      <c r="AN10" t="s">
+        <v>177</v>
+      </c>
+      <c r="AO10" t="s">
+        <v>177</v>
+      </c>
+      <c r="AP10" t="s">
+        <v>177</v>
+      </c>
+      <c r="AQ10" t="s">
+        <v>177</v>
+      </c>
+      <c r="AR10" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="11" spans="1:47">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C11" t="s">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="D11" t="s">
-        <v>109</v>
+        <v>124</v>
       </c>
       <c r="E11" t="s">
-        <v>135</v>
+        <v>156</v>
       </c>
       <c r="F11" t="s">
-        <v>147</v>
+        <v>174</v>
       </c>
       <c r="G11" t="s">
-        <v>149</v>
+        <v>176</v>
       </c>
       <c r="H11" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="I11" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="J11" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="K11" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="L11" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="M11" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="N11" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="O11" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="P11" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="Q11" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="R11" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="S11" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="T11" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="U11" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="V11" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="W11" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="X11" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="Y11" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="Z11" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AA11" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AB11" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AC11" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AD11" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AE11" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AF11" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AG11" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AH11" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AI11" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AJ11" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AK11" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AL11" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AM11" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AN11" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AO11" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AP11" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AQ11" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AR11" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="12" spans="1:44">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="12" spans="1:47">
       <c r="A12">
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="C12" t="s">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="D12" t="s">
-        <v>110</v>
+        <v>125</v>
       </c>
       <c r="E12" t="s">
-        <v>136</v>
+        <v>157</v>
       </c>
       <c r="F12" t="s">
-        <v>147</v>
+        <v>174</v>
       </c>
       <c r="G12" t="s">
-        <v>149</v>
+        <v>176</v>
       </c>
       <c r="H12" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="I12" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="J12" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="K12" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="L12" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="M12" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="N12" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="O12" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="P12" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="Q12" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="R12" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="S12" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="T12" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="U12" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="V12" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="W12" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="X12" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="Y12" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="Z12" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AA12" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AB12" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AC12" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AD12" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AE12" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AF12" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AG12" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AH12" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AI12" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AJ12" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AK12" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AL12" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AM12" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AN12" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AO12" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AP12" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AQ12" t="s">
-        <v>150</v>
-      </c>
-      <c r="AR12" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="13" spans="1:44">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="13" spans="1:47">
       <c r="A13">
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C13" t="s">
-        <v>83</v>
+        <v>92</v>
       </c>
       <c r="D13" t="s">
-        <v>111</v>
+        <v>126</v>
       </c>
       <c r="E13" t="s">
-        <v>137</v>
+        <v>158</v>
       </c>
       <c r="F13" t="s">
-        <v>147</v>
+        <v>174</v>
       </c>
       <c r="G13" t="s">
-        <v>149</v>
+        <v>176</v>
       </c>
       <c r="H13" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="I13" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="J13" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="K13" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="L13" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="M13" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="N13" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="O13" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="P13" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="Q13" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="R13" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="S13" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="T13" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="U13" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="V13" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="W13" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="X13" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="Y13" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="Z13" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AA13" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AB13" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AC13" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AD13" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AE13" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AF13" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AG13" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AH13" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AI13" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AJ13" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AK13" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AL13" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AM13" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AN13" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AO13" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AP13" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AQ13" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AR13" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="14" spans="1:44">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="14" spans="1:47">
       <c r="A14">
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="C14" t="s">
-        <v>84</v>
+        <v>93</v>
       </c>
       <c r="D14" t="s">
-        <v>112</v>
+        <v>127</v>
       </c>
       <c r="E14" t="s">
-        <v>138</v>
+        <v>159</v>
       </c>
       <c r="F14" t="s">
-        <v>147</v>
+        <v>174</v>
       </c>
       <c r="G14" t="s">
-        <v>149</v>
+        <v>176</v>
       </c>
       <c r="H14" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="I14" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="J14" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="K14" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="L14" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="M14" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="N14" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="O14" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="P14" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="Q14" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="R14" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="S14" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="T14" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="U14" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="V14" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="W14" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="X14" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="Y14" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="Z14" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AA14" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AB14" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AC14" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AD14" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AE14" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AF14" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AG14" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AH14" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AI14" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AJ14" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AK14" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AL14" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AM14" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AN14" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AO14" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AP14" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AQ14" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AR14" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="15" spans="1:44">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="15" spans="1:47">
       <c r="A15">
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C15" t="s">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="D15" t="s">
-        <v>113</v>
+        <v>128</v>
       </c>
       <c r="E15" t="s">
-        <v>139</v>
+        <v>160</v>
       </c>
       <c r="F15" t="s">
-        <v>147</v>
+        <v>174</v>
       </c>
       <c r="G15" t="s">
-        <v>149</v>
+        <v>176</v>
       </c>
       <c r="H15" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="I15" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="J15" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="K15" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="L15" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="M15" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="N15" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="O15" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="P15" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="Q15" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="R15" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="S15" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="T15" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="U15" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="V15" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="W15" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="X15" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="Y15" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="Z15" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AA15" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AB15" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AC15" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AD15" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AE15" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AF15" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AG15" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AH15" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AI15" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AJ15" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AK15" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AL15" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AM15" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AN15" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AO15" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AP15" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AQ15" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AR15" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="16" spans="1:44">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="16" spans="1:47">
       <c r="A16">
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C16" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="D16" t="s">
-        <v>114</v>
+        <v>129</v>
       </c>
       <c r="E16" t="s">
-        <v>129</v>
+        <v>150</v>
       </c>
       <c r="F16" t="s">
-        <v>148</v>
+        <v>175</v>
       </c>
       <c r="G16" t="s">
-        <v>149</v>
+        <v>176</v>
       </c>
       <c r="O16" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="P16" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
     </row>
     <row r="17" spans="1:44">
@@ -2013,133 +2325,133 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C17" t="s">
-        <v>87</v>
+        <v>96</v>
       </c>
       <c r="D17" t="s">
-        <v>115</v>
+        <v>130</v>
       </c>
       <c r="E17" t="s">
-        <v>140</v>
+        <v>161</v>
       </c>
       <c r="F17" t="s">
-        <v>147</v>
+        <v>174</v>
       </c>
       <c r="G17" t="s">
-        <v>149</v>
+        <v>176</v>
       </c>
       <c r="H17" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="I17" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="J17" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="K17" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="L17" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="M17" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="N17" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="O17" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="P17" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="Q17" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="R17" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="S17" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="T17" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="U17" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="V17" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="W17" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="X17" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="Y17" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="Z17" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AA17" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AB17" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AC17" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AD17" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AE17" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AF17" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AG17" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AH17" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AI17" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AJ17" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AK17" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AL17" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AM17" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AN17" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AO17" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AP17" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AQ17" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="AR17" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
     </row>
     <row r="18" spans="1:44">
@@ -2147,28 +2459,28 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C18" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="D18" t="s">
-        <v>116</v>
+        <v>131</v>
       </c>
       <c r="E18" t="s">
-        <v>131</v>
+        <v>152</v>
       </c>
       <c r="F18" t="s">
-        <v>147</v>
+        <v>174</v>
       </c>
       <c r="G18" t="s">
-        <v>149</v>
+        <v>176</v>
       </c>
       <c r="O18" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
       <c r="P18" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
     </row>
     <row r="19" spans="1:44">
@@ -2176,25 +2488,25 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="C19" t="s">
-        <v>89</v>
+        <v>98</v>
       </c>
       <c r="D19" t="s">
-        <v>117</v>
+        <v>132</v>
       </c>
       <c r="E19" t="s">
-        <v>129</v>
+        <v>150</v>
       </c>
       <c r="F19" t="s">
-        <v>148</v>
+        <v>175</v>
       </c>
       <c r="G19" t="s">
-        <v>149</v>
+        <v>176</v>
       </c>
       <c r="I19" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
     </row>
     <row r="20" spans="1:44">
@@ -2202,25 +2514,25 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C20" t="s">
-        <v>90</v>
+        <v>99</v>
       </c>
       <c r="D20" t="s">
-        <v>118</v>
+        <v>133</v>
       </c>
       <c r="E20" t="s">
-        <v>129</v>
+        <v>150</v>
       </c>
       <c r="F20" t="s">
-        <v>148</v>
+        <v>175</v>
       </c>
       <c r="G20" t="s">
-        <v>149</v>
+        <v>176</v>
       </c>
       <c r="K20" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
     </row>
     <row r="21" spans="1:44">
@@ -2228,25 +2540,25 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="C21" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="D21" t="s">
-        <v>119</v>
+        <v>134</v>
       </c>
       <c r="E21" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="F21" t="s">
-        <v>147</v>
+        <v>174</v>
       </c>
       <c r="G21" t="s">
-        <v>149</v>
+        <v>176</v>
       </c>
       <c r="P21" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
     </row>
     <row r="22" spans="1:44">
@@ -2254,25 +2566,25 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="C22" t="s">
-        <v>92</v>
+        <v>101</v>
       </c>
       <c r="D22" t="s">
-        <v>120</v>
+        <v>135</v>
       </c>
       <c r="E22" t="s">
-        <v>142</v>
+        <v>163</v>
       </c>
       <c r="F22" t="s">
-        <v>147</v>
+        <v>174</v>
       </c>
       <c r="G22" t="s">
-        <v>149</v>
+        <v>176</v>
       </c>
       <c r="X22" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
     </row>
     <row r="23" spans="1:44">
@@ -2280,28 +2592,31 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="C23" t="s">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="D23" t="s">
-        <v>121</v>
+        <v>136</v>
       </c>
       <c r="E23" t="s">
-        <v>143</v>
+        <v>164</v>
       </c>
       <c r="F23" t="s">
-        <v>147</v>
+        <v>174</v>
       </c>
       <c r="G23" t="s">
-        <v>149</v>
+        <v>176</v>
       </c>
       <c r="M23" t="s">
-        <v>150</v>
+        <v>177</v>
+      </c>
+      <c r="AA23" t="s">
+        <v>177</v>
       </c>
       <c r="AC23" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
     </row>
     <row r="24" spans="1:44">
@@ -2309,25 +2624,25 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C24" t="s">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="D24" t="s">
-        <v>122</v>
+        <v>137</v>
       </c>
       <c r="E24" t="s">
-        <v>144</v>
+        <v>165</v>
       </c>
       <c r="F24" t="s">
-        <v>147</v>
+        <v>174</v>
       </c>
       <c r="G24" t="s">
-        <v>149</v>
+        <v>176</v>
       </c>
       <c r="AE24" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
     </row>
     <row r="25" spans="1:44">
@@ -2335,25 +2650,25 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C25" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="D25" t="s">
-        <v>123</v>
+        <v>138</v>
       </c>
       <c r="E25" t="s">
-        <v>129</v>
+        <v>150</v>
       </c>
       <c r="F25" t="s">
-        <v>148</v>
+        <v>175</v>
       </c>
       <c r="G25" t="s">
-        <v>149</v>
+        <v>176</v>
       </c>
       <c r="P25" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
     </row>
     <row r="26" spans="1:44">
@@ -2361,25 +2676,25 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="C26" t="s">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="D26" t="s">
-        <v>124</v>
+        <v>139</v>
       </c>
       <c r="E26" t="s">
-        <v>129</v>
+        <v>150</v>
       </c>
       <c r="F26" t="s">
-        <v>148</v>
+        <v>175</v>
       </c>
       <c r="G26" t="s">
-        <v>149</v>
+        <v>176</v>
       </c>
       <c r="P26" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
     </row>
     <row r="27" spans="1:44">
@@ -2387,25 +2702,25 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C27" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="D27" t="s">
-        <v>125</v>
+        <v>140</v>
       </c>
       <c r="E27" t="s">
-        <v>145</v>
+        <v>166</v>
       </c>
       <c r="F27" t="s">
-        <v>147</v>
+        <v>174</v>
       </c>
       <c r="G27" t="s">
-        <v>149</v>
+        <v>176</v>
       </c>
       <c r="P27" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
     </row>
     <row r="28" spans="1:44">
@@ -2413,25 +2728,25 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="C28" t="s">
-        <v>98</v>
+        <v>107</v>
       </c>
       <c r="D28" t="s">
-        <v>126</v>
+        <v>141</v>
       </c>
       <c r="E28" t="s">
-        <v>145</v>
+        <v>166</v>
       </c>
       <c r="F28" t="s">
-        <v>147</v>
+        <v>174</v>
       </c>
       <c r="G28" t="s">
-        <v>149</v>
+        <v>176</v>
       </c>
       <c r="P28" t="s">
-        <v>150</v>
+        <v>177</v>
       </c>
     </row>
     <row r="29" spans="1:44">
@@ -2439,25 +2754,139 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="C29" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="D29" t="s">
-        <v>127</v>
+        <v>142</v>
       </c>
       <c r="E29" t="s">
+        <v>167</v>
+      </c>
+      <c r="F29" t="s">
+        <v>174</v>
+      </c>
+      <c r="G29" t="s">
+        <v>176</v>
+      </c>
+      <c r="P29" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="30" spans="1:44">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" t="s">
+        <v>75</v>
+      </c>
+      <c r="C30" t="s">
+        <v>109</v>
+      </c>
+      <c r="D30" t="s">
+        <v>143</v>
+      </c>
+      <c r="E30" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="31" spans="1:44">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31" t="s">
+        <v>76</v>
+      </c>
+      <c r="C31" t="s">
+        <v>110</v>
+      </c>
+      <c r="D31" t="s">
+        <v>144</v>
+      </c>
+      <c r="E31" t="s">
+        <v>169</v>
+      </c>
+      <c r="AR31" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="32" spans="1:44">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32" t="s">
+        <v>77</v>
+      </c>
+      <c r="C32" t="s">
+        <v>111</v>
+      </c>
+      <c r="D32" t="s">
+        <v>145</v>
+      </c>
+      <c r="E32" t="s">
+        <v>170</v>
+      </c>
+      <c r="AD32" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="33" spans="1:28">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33" t="s">
+        <v>78</v>
+      </c>
+      <c r="C33" t="s">
+        <v>112</v>
+      </c>
+      <c r="D33" t="s">
         <v>146</v>
       </c>
-      <c r="F29" t="s">
+      <c r="E33" t="s">
+        <v>171</v>
+      </c>
+      <c r="Z33" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="34" spans="1:28">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34" t="s">
+        <v>79</v>
+      </c>
+      <c r="C34" t="s">
+        <v>113</v>
+      </c>
+      <c r="D34" t="s">
         <v>147</v>
       </c>
-      <c r="G29" t="s">
-        <v>149</v>
-      </c>
-      <c r="P29" t="s">
-        <v>150</v>
+      <c r="E34" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="35" spans="1:28">
+      <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35" t="s">
+        <v>80</v>
+      </c>
+      <c r="C35" t="s">
+        <v>114</v>
+      </c>
+      <c r="D35" t="s">
+        <v>148</v>
+      </c>
+      <c r="E35" t="s">
+        <v>173</v>
+      </c>
+      <c r="AB35" t="s">
+        <v>177</v>
       </c>
     </row>
   </sheetData>

</xml_diff>